<commit_message>
Expand elec sources used for least cost dispatch
</commit_message>
<xml_diff>
--- a/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
+++ b/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todd/eps/eps-us/InputData/elec/ESUfRaLCD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\ESUfRaLCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26578C50-7F18-C947-84CA-18CC1CD39ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD736FDD-8F83-4A21-879A-10EA011AD972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="67">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -187,15 +187,9 @@
     <t>biomass</t>
   </si>
   <si>
-    <t>biomass dispatch</t>
-  </si>
-  <si>
     <t>hydro</t>
   </si>
   <si>
-    <t>hydro dispatch</t>
-  </si>
-  <si>
     <t>hard coal w ccs es</t>
   </si>
   <si>
@@ -212,13 +206,43 @@
   </si>
   <si>
     <t>lignite w ccs</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>solar thermal</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>offshore wind</t>
+  </si>
+  <si>
+    <t>crude oil</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
+  </si>
+  <si>
+    <t>hard coal w CCS</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle w CCS</t>
+  </si>
+  <si>
+    <t>biomass w CCS</t>
+  </si>
+  <si>
+    <t>lignite w CCS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,6 +261,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -262,10 +293,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,14 +615,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -596,7 +630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -604,142 +638,142 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -755,13 +789,13 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:C84"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="30.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -772,7 +806,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -785,7 +819,7 @@
         <v>natural gas combined cycle power plants</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -798,7 +832,7 @@
         <v>onshore wind power plants</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -811,7 +845,7 @@
         <v>solar PV power plants</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -824,7 +858,7 @@
         <v>petroleum power plants</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -837,7 +871,7 @@
         <v>natural gas peaker power plants</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -850,33 +884,33 @@
         <v>small modular reactor power plants</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="1"/>
+        <v>hard coal w ccs power plants</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>natural gas combined cycle w ccs power plants</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>55</v>
-      </c>
-      <c r="B8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="1"/>
-        <v>hard coal w ccs power plants</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="1"/>
-        <v>natural gas combined cycle w ccs power plants</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>57</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
@@ -886,9 +920,9 @@
         <v>biomass w ccs power plants</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
@@ -898,7 +932,7 @@
         <v>lignite w ccs power plants</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -911,7 +945,7 @@
         <v>hydrogen combustion turbine power plants</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -924,7 +958,7 @@
         <v>hydrogen combined cycle power plants</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -934,7 +968,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -944,7 +978,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -954,7 +988,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -964,7 +998,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -974,7 +1008,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -984,7 +1018,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -994,7 +1028,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1004,7 +1038,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1014,7 +1048,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1024,7 +1058,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1034,7 +1068,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1044,355 +1078,355 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C26" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C29" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C32" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C34" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C35" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C36" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C37" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C38" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C39" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C40" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C41" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C42" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C43" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C44" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C45" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C47" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C48" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C49" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C50" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C51" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C52" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C53" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C54" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C55" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C56" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C57" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C58" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C59" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C60" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C61" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C62" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C63" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C64" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C65" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C66" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C67" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C68" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C69" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C70" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C71" t="str">
         <f t="shared" ref="C71:C84" si="2">IF(A71="","",CONCATENATE(A71," power plants"))</f>
         <v/>
       </c>
     </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C72" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C73" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C74" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C75" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C76" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C77" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C78" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C79" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="80" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C80" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C81" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="82" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C82" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="83" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C83" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="84" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C84" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -1408,14 +1442,14 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1426,7 +1460,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1439,20 +1473,20 @@
         <v>hard coal dispatch</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>44</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B17" si="0">IF(A3="","",CONCATENATE(A3," es"))</f>
+        <f t="shared" ref="B3:B25" si="0">IF(A3="","",CONCATENATE(A3," es"))</f>
         <v>natural gas steam turbine es</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C17" si="1">IF(A3="","",CONCATENATE(A3," dispatch"))</f>
+        <f t="shared" ref="C3:C25" si="1">IF(A3="","",CONCATENATE(A3," dispatch"))</f>
         <v>natural gas steam turbine dispatch</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1465,163 +1499,275 @@
         <v>natural gas combined cycle dispatch</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>nuclear es</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="1"/>
+        <v>nuclear dispatch</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>hydro es</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="1"/>
+        <v>hydro dispatch</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>onshore wind es</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="1"/>
+        <v>onshore wind dispatch</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>solar PV es</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="1"/>
+        <v>solar PV dispatch</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>solar thermal es</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>solar thermal dispatch</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass es</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="1"/>
+        <v>biomass dispatch</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>geothermal es</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="1"/>
+        <v>geothermal dispatch</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>32</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>petroleum es</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C12" t="str">
         <f t="shared" si="1"/>
         <v>petroleum dispatch</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>33</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>natural gas peaker es</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C13" t="str">
         <f t="shared" si="1"/>
         <v>natural gas peaker dispatch</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>lignite es</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C14" t="str">
         <f t="shared" si="1"/>
         <v>lignite dispatch</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>offshore wind es</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>offshore wind dispatch</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>crude oil es</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>crude oil dispatch</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>heavy or residual fuel oil es</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="1"/>
+        <v>heavy or residual fuel oil dispatch</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>46</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>municipal solid waste es</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C18" t="str">
         <f t="shared" si="1"/>
         <v>municipal solid waste dispatch</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" t="str">
-        <f t="shared" si="1"/>
-        <v>hard coal w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" t="str">
-        <f t="shared" si="1"/>
-        <v>natural gas combined cycle w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="str">
-        <f t="shared" si="1"/>
-        <v>biomass w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="str">
-        <f t="shared" si="1"/>
-        <v>lignite w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>hard coal w CCS es</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>hard coal w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>natural gas combined cycle w CCS es</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>natural gas combined cycle w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass w CCS es</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>biomass w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>lignite w CCS es</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="1"/>
+        <v>lignite w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>34</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>small modular reactor es</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C23" t="str">
         <f t="shared" si="1"/>
         <v>small modular reactor dispatch</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>hydrogen combustion turbine es</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C24" t="str">
         <f t="shared" si="1"/>
         <v>hydrogen combustion turbine dispatch</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>hydrogen combined cycle es</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C25" t="str">
         <f t="shared" si="1"/>
         <v>hydrogen combined cycle dispatch</v>
       </c>

</xml_diff>

<commit_message>
Correct subscript mapping in the ESUfRaLCD file
</commit_message>
<xml_diff>
--- a/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
+++ b/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\ESUfRaLCD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\ESUfRaLCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC20DFE0-FCA2-41EA-B845-0C40661B8AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB1025B6-1BC7-4047-9FEE-D6C084499EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="5700" windowWidth="43200" windowHeight="17145" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="61">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -188,12 +188,6 @@
   </si>
   <si>
     <t>hydro</t>
-  </si>
-  <si>
-    <t>hard coal w ccs es</t>
-  </si>
-  <si>
-    <t>natural gas combined cycle w ccs es</t>
   </si>
   <si>
     <t>nuclear</t>
@@ -593,14 +587,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -608,7 +602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -616,142 +610,142 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -767,13 +761,13 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:C84"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="30.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -784,7 +778,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -793,11 +787,11 @@
         <v>hard coal es</v>
       </c>
       <c r="C2" t="str">
-        <f>IF(A2="","",CONCATENATE(A2," power plants"))</f>
-        <v>hard coal power plants</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <f>IF(A2="","",CONCATENATE(A2," dispatch"))</f>
+        <v>hard coal dispatch</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -806,11 +800,11 @@
         <v>natural gas steam turbine es</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C70" si="1">IF(A3="","",CONCATENATE(A3," power plants"))</f>
-        <v>natural gas steam turbine power plants</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" ref="C3:C25" si="1">IF(A3="","",CONCATENATE(A3," dispatch"))</f>
+        <v>natural gas steam turbine dispatch</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -820,12 +814,12 @@
       </c>
       <c r="C4" t="str">
         <f t="shared" si="1"/>
-        <v>natural gas combined cycle power plants</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>natural gas combined cycle dispatch</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -833,10 +827,10 @@
       </c>
       <c r="C5" t="str">
         <f t="shared" si="1"/>
-        <v>nuclear power plants</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>nuclear dispatch</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -845,11 +839,11 @@
         <v>hydro es</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="1"/>
-        <v>hydro power plants</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <f>IF(A6="","",CONCATENATE(A6," dispatch"))</f>
+        <v>hydro dispatch</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -859,58 +853,62 @@
       </c>
       <c r="C7" t="str">
         <f t="shared" si="1"/>
-        <v>onshore wind power plants</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>onshore wind dispatch</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>31</v>
       </c>
-      <c r="B8" t="s">
-        <v>51</v>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>solar PV es</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
-        <v>solar PV power plants</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>solar PV dispatch</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" t="s">
         <v>52</v>
       </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>solar thermal es</v>
+      </c>
       <c r="C9" t="str">
         <f t="shared" si="1"/>
-        <v>solar thermal power plants</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>solar thermal dispatch</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B10" t="s">
-        <v>25</v>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass es</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="1"/>
-        <v>biomass power plants</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>biomass dispatch</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" t="s">
-        <v>26</v>
+        <v>53</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>geothermal es</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="1"/>
-        <v>geothermal power plants</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>geothermal dispatch</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -920,10 +918,10 @@
       </c>
       <c r="C12" t="str">
         <f t="shared" si="1"/>
-        <v>petroleum power plants</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>petroleum dispatch</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -933,10 +931,10 @@
       </c>
       <c r="C13" t="str">
         <f t="shared" si="1"/>
-        <v>natural gas peaker power plants</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>natural gas peaker dispatch</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -946,49 +944,49 @@
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
-        <v>lignite power plants</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>lignite dispatch</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>offshore wind es</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>offshore wind dispatch</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>crude oil es</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>crude oil dispatch</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>56</v>
       </c>
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v>offshore wind es</v>
-      </c>
-      <c r="C15" t="str">
-        <f t="shared" si="1"/>
-        <v>offshore wind power plants</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>crude oil es</v>
-      </c>
-      <c r="C16" t="str">
-        <f t="shared" si="1"/>
-        <v>crude oil power plants</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>58</v>
-      </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>heavy or residual fuel oil es</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="1"/>
-        <v>heavy or residual fuel oil power plants</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>heavy or residual fuel oil dispatch</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -998,62 +996,62 @@
       </c>
       <c r="C18" t="str">
         <f t="shared" si="1"/>
-        <v>municipal solid waste power plants</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>municipal solid waste dispatch</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>hard coal w CCS es</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>hard coal w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>natural gas combined cycle w CCS es</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>natural gas combined cycle w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>59</v>
       </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>hard coal w CCS es</v>
-      </c>
-      <c r="C19" t="str">
-        <f t="shared" si="1"/>
-        <v>hard coal w CCS power plants</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass w CCS es</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>biomass w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>60</v>
       </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>natural gas combined cycle w CCS es</v>
-      </c>
-      <c r="C20" t="str">
-        <f t="shared" si="1"/>
-        <v>natural gas combined cycle w CCS power plants</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>biomass w CCS es</v>
-      </c>
-      <c r="C21" t="str">
-        <f t="shared" si="1"/>
-        <v>biomass w CCS power plants</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>lignite w CCS es</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="1"/>
-        <v>lignite w CCS power plants</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>lignite w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -1063,10 +1061,10 @@
       </c>
       <c r="C23" t="str">
         <f t="shared" si="1"/>
-        <v>small modular reactor power plants</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>small modular reactor dispatch</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -1076,10 +1074,10 @@
       </c>
       <c r="C24" t="str">
         <f t="shared" si="1"/>
-        <v>hydrogen combustion turbine power plants</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>hydrogen combustion turbine dispatch</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -1089,360 +1087,360 @@
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>hydrogen combined cycle power plants</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>hydrogen combined cycle dispatch</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" ref="C3:C70" si="2">IF(A26="","",CONCATENATE(A26," power plants"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C27" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C28" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C30" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C31" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C32" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C33" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C34" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C35" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C36" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C37" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C38" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C39" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C40" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C41" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C42" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C43" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C44" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C45" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C46" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C47" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C48" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C49" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C50" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C51" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C52" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C53" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C54" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C55" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C56" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C57" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C58" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C59" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C60" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C61" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C62" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C63" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C64" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C65" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C66" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C67" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C68" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C69" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C70" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C71" t="str">
-        <f t="shared" ref="C71:C84" si="2">IF(A71="","",CONCATENATE(A71," power plants"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" ref="C71:C84" si="3">IF(A71="","",CONCATENATE(A71," power plants"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C72" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C73" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C74" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C75" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C76" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C77" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C78" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C79" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C80" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C81" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C82" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C83" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C84" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -1457,13 +1455,13 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1474,7 +1472,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1487,7 +1485,7 @@
         <v>hard coal dispatch</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1500,7 +1498,7 @@
         <v>natural gas steam turbine dispatch</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1513,9 +1511,9 @@
         <v>natural gas combined cycle dispatch</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -1526,7 +1524,7 @@
         <v>nuclear dispatch</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -1539,7 +1537,7 @@
         <v>hydro dispatch</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1552,7 +1550,7 @@
         <v>onshore wind dispatch</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -1565,9 +1563,9 @@
         <v>solar PV dispatch</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -1578,7 +1576,7 @@
         <v>solar thermal dispatch</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -1591,9 +1589,9 @@
         <v>biomass dispatch</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -1604,7 +1602,7 @@
         <v>geothermal dispatch</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1617,7 +1615,7 @@
         <v>petroleum dispatch</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1630,7 +1628,7 @@
         <v>natural gas peaker dispatch</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1643,36 +1641,36 @@
         <v>lignite dispatch</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>offshore wind es</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>offshore wind dispatch</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>crude oil es</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>crude oil dispatch</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>56</v>
       </c>
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v>offshore wind es</v>
-      </c>
-      <c r="C15" t="str">
-        <f t="shared" si="1"/>
-        <v>offshore wind dispatch</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>crude oil es</v>
-      </c>
-      <c r="C16" t="str">
-        <f t="shared" si="1"/>
-        <v>crude oil dispatch</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>58</v>
-      </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>heavy or residual fuel oil es</v>
@@ -1682,7 +1680,7 @@
         <v>heavy or residual fuel oil dispatch</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -1695,49 +1693,49 @@
         <v>municipal solid waste dispatch</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>hard coal w CCS es</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>hard coal w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>natural gas combined cycle w CCS es</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>natural gas combined cycle w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>59</v>
       </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>hard coal w CCS es</v>
-      </c>
-      <c r="C19" t="str">
-        <f t="shared" si="1"/>
-        <v>hard coal w CCS dispatch</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass w CCS es</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>biomass w CCS dispatch</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>60</v>
       </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>natural gas combined cycle w CCS es</v>
-      </c>
-      <c r="C20" t="str">
-        <f t="shared" si="1"/>
-        <v>natural gas combined cycle w CCS dispatch</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>biomass w CCS es</v>
-      </c>
-      <c r="C21" t="str">
-        <f t="shared" si="1"/>
-        <v>biomass w CCS dispatch</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>lignite w CCS es</v>
@@ -1747,7 +1745,7 @@
         <v>lignite w CCS dispatch</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -1760,7 +1758,7 @@
         <v>small modular reactor dispatch</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -1773,7 +1771,7 @@
         <v>hydrogen combustion turbine dispatch</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>36</v>
       </c>

</xml_diff>